<commit_message>
fix: atualiza planilha CONTAS-A-RECEBER (61 vencidos, R$ 28.296,02)
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planilhas/CONTAS-A-RECEBER.xlsx
+++ b/planilhas/CONTAS-A-RECEBER.xlsx
@@ -9,14 +9,14 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Relatório!$A$5:$S$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Relatório!$A$1:$S$30</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Relatório!$A$1:$S$106</definedName>
   </definedNames>
   <calcPr fullCalcOnLoad="1" fullPrecision="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="163">
   <si>
     <t>Contas a Receber em aberto</t>
   </si>
@@ -36,7 +36,7 @@
         <color rgb="FF808080"/>
         <sz val="11"/>
       </rPr>
-      <t>Data Final: 07/06/2026</t>
+      <t>Data Inicial: 01/04/2026, Data Final: 15/06/2026</t>
     </r>
   </si>
   <si>
@@ -209,6 +209,318 @@
   </si>
   <si>
     <t>OLIZIEL DA SILVA CARDOSO</t>
+  </si>
+  <si>
+    <t>ND-11699</t>
+  </si>
+  <si>
+    <t>ROSSILY PEREIRA DA SILVA</t>
+  </si>
+  <si>
+    <t>PRIVADO</t>
+  </si>
+  <si>
+    <t>ND-11700</t>
+  </si>
+  <si>
+    <t>JOAO PAULO CONSORCIOS</t>
+  </si>
+  <si>
+    <t>JOAO PAULO SERVICOS DE CONSULTORIA EM CONSORCIOS LTDA</t>
+  </si>
+  <si>
+    <t>LUZ DIVINA LOCACAO DE ATIVOS</t>
+  </si>
+  <si>
+    <t>LUZ DIVINA EMPREENDIMENTOS LTDA</t>
+  </si>
+  <si>
+    <t>FA-11617</t>
+  </si>
+  <si>
+    <t>FA-11709</t>
+  </si>
+  <si>
+    <t>FA-11717</t>
+  </si>
+  <si>
+    <t>ADRIANO SANTOS DE CARVALHO</t>
+  </si>
+  <si>
+    <t>FA-11692</t>
+  </si>
+  <si>
+    <t>FA-11774</t>
+  </si>
+  <si>
+    <t>DERICK PEDRO BEZERRA DA ROCHA</t>
+  </si>
+  <si>
+    <t>FA-11784</t>
+  </si>
+  <si>
+    <t>FA-11569</t>
+  </si>
+  <si>
+    <t>FA-11568</t>
+  </si>
+  <si>
+    <t>FA-11796</t>
+  </si>
+  <si>
+    <t>FA-11685</t>
+  </si>
+  <si>
+    <t>GILVAN RODRIGUES MACHADO</t>
+  </si>
+  <si>
+    <t>FA-11720</t>
+  </si>
+  <si>
+    <t>FA-11670</t>
+  </si>
+  <si>
+    <t>RICARDO ARAUJO DE MIRANDA</t>
+  </si>
+  <si>
+    <t>FA-11775</t>
+  </si>
+  <si>
+    <t>FA-11795</t>
+  </si>
+  <si>
+    <t>FELIPE DA SILVA</t>
+  </si>
+  <si>
+    <t>FA-11693</t>
+  </si>
+  <si>
+    <t>FA-11570</t>
+  </si>
+  <si>
+    <t>ELSON VIEIRA DA SILVA</t>
+  </si>
+  <si>
+    <t>FA-11815</t>
+  </si>
+  <si>
+    <t>LEONARDO GOMES DO NASCIMENTO</t>
+  </si>
+  <si>
+    <t>FA-11814</t>
+  </si>
+  <si>
+    <t>FA-11678</t>
+  </si>
+  <si>
+    <t>FA-11782</t>
+  </si>
+  <si>
+    <t>FERNANDO RODRIGUES DO NASCIMENTO</t>
+  </si>
+  <si>
+    <t>FA-11763</t>
+  </si>
+  <si>
+    <t>ANNY KATARINA ACIOLE DA SILVA</t>
+  </si>
+  <si>
+    <t>Z. FROTA INVESTIDORES - JOÃO PAULO</t>
+  </si>
+  <si>
+    <t>FA-11816</t>
+  </si>
+  <si>
+    <t>ELIONILSON CORDEIRO BARBOSA</t>
+  </si>
+  <si>
+    <t>JOÃO PAULO CONSÓRCIOS</t>
+  </si>
+  <si>
+    <t>FA-11603</t>
+  </si>
+  <si>
+    <t>PEDRO GABRIEL FASANARO DE OLIVEIRA</t>
+  </si>
+  <si>
+    <t>FA-11593</t>
+  </si>
+  <si>
+    <t>JACKSON CASSIANO VERISSIMO</t>
+  </si>
+  <si>
+    <t>LUZ DIVINA LTDA</t>
+  </si>
+  <si>
+    <t>ND-11801</t>
+  </si>
+  <si>
+    <t>FA-11755</t>
+  </si>
+  <si>
+    <t>MARIO EWERTON CANDIDO DE SOUZA</t>
+  </si>
+  <si>
+    <t>HOJE</t>
+  </si>
+  <si>
+    <t>FA-11805</t>
+  </si>
+  <si>
+    <t>RAFAEL CAVALCANTI BARROS FERREIRA</t>
+  </si>
+  <si>
+    <t>FA-11813</t>
+  </si>
+  <si>
+    <t>ANDERSON QUEIROZ PINHEIRO</t>
+  </si>
+  <si>
+    <t>A VENCER</t>
+  </si>
+  <si>
+    <t>FA-11748</t>
+  </si>
+  <si>
+    <t>ROBERTO MURATORI</t>
+  </si>
+  <si>
+    <t>FA-11787</t>
+  </si>
+  <si>
+    <t>FA-11726</t>
+  </si>
+  <si>
+    <t>JOZILDO TARQUINO DE BRITO</t>
+  </si>
+  <si>
+    <t>FA-11572</t>
+  </si>
+  <si>
+    <t>FA-11806</t>
+  </si>
+  <si>
+    <t>FA-11571</t>
+  </si>
+  <si>
+    <t>FA-11786</t>
+  </si>
+  <si>
+    <t>FA-11798</t>
+  </si>
+  <si>
+    <t>FA-11686</t>
+  </si>
+  <si>
+    <t>FA-11756</t>
+  </si>
+  <si>
+    <t>FA-11671</t>
+  </si>
+  <si>
+    <t>FA-11729</t>
+  </si>
+  <si>
+    <t>JONILSON JOSEMAR DO NASCIMENTO</t>
+  </si>
+  <si>
+    <t>FA-11724</t>
+  </si>
+  <si>
+    <t>FA-11727</t>
+  </si>
+  <si>
+    <t>ANA FLORIPES CARVALHO DA CUNHA</t>
+  </si>
+  <si>
+    <t>FA-11776</t>
+  </si>
+  <si>
+    <t>FA-11659</t>
+  </si>
+  <si>
+    <t>LUCA ZOLI</t>
+  </si>
+  <si>
+    <t>FA-11624</t>
+  </si>
+  <si>
+    <t>DANILO DE ALMEIDA TORRES</t>
+  </si>
+  <si>
+    <t>FA-11797</t>
+  </si>
+  <si>
+    <t>FA-11507</t>
+  </si>
+  <si>
+    <t>WESCLY JEAN DE MEDEIROS</t>
+  </si>
+  <si>
+    <t>FA-11437</t>
+  </si>
+  <si>
+    <t>RAYANE ROBERTA DA SILVA</t>
+  </si>
+  <si>
+    <t>FA-11694</t>
+  </si>
+  <si>
+    <t>FA-11810</t>
+  </si>
+  <si>
+    <t>LUCAS NAJA MOURA RODRIGUES</t>
+  </si>
+  <si>
+    <t>FA-11819</t>
+  </si>
+  <si>
+    <t>FA-11573</t>
+  </si>
+  <si>
+    <t>FA-11817</t>
+  </si>
+  <si>
+    <t>FA-11679</t>
+  </si>
+  <si>
+    <t>FA-11818</t>
+  </si>
+  <si>
+    <t>FA-11785</t>
+  </si>
+  <si>
+    <t>FA-11764</t>
+  </si>
+  <si>
+    <t>FA-11604</t>
+  </si>
+  <si>
+    <t>FA-11820</t>
+  </si>
+  <si>
+    <t>FA-11581</t>
+  </si>
+  <si>
+    <t>ADRIANO TEOTONIO DA SILVA</t>
+  </si>
+  <si>
+    <t>FA-11635</t>
+  </si>
+  <si>
+    <t>TANIELLE GLAUCIANA SOUZA DA SILVA</t>
+  </si>
+  <si>
+    <t>PÚBLICO</t>
+  </si>
+  <si>
+    <t>FA-11594</t>
+  </si>
+  <si>
+    <t>FA-11647</t>
+  </si>
+  <si>
+    <t>MARCIANO EZEQUIEL VALDEVINO DA SILVA</t>
   </si>
 </sst>
 </file>
@@ -351,7 +663,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr codeName=""/>
-  <dimension ref="A1:S30"/>
+  <dimension ref="A1:S106"/>
   <sheetFormatPr defaultRowHeight="23" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="38" customWidth="1" style="1"/>
@@ -366,12 +678,12 @@
     <col min="10" max="10" width="21" customWidth="1" style="1"/>
     <col min="11" max="11" width="13" customWidth="1" style="1"/>
     <col min="12" max="12" width="39" customWidth="1" style="1"/>
-    <col min="13" max="13" width="27" customWidth="1" style="1"/>
+    <col min="13" max="13" width="55" customWidth="1" style="1"/>
     <col min="14" max="14" width="31" customWidth="1" style="1"/>
     <col min="15" max="15" width="26" customWidth="1" style="1"/>
     <col min="16" max="16" width="14" customWidth="1" style="1"/>
     <col min="17" max="17" width="16" customWidth="1" style="1"/>
-    <col min="18" max="18" width="20" customWidth="1" style="1"/>
+    <col min="18" max="18" width="23" customWidth="1" style="1"/>
     <col min="19" max="19" width="16" customWidth="1" style="1"/>
     <col min="20" max="16384" width="9.140625" customWidth="1" style="1"/>
   </cols>
@@ -1867,27 +2179,4511 @@
         <v>680</v>
       </c>
     </row>
-    <row r="30" ht="23" customHeight="1">
-      <c r="A30" s="10"/>
-      <c r="B30" s="11"/>
-      <c r="C30" s="11"/>
-      <c r="D30" s="11"/>
-      <c r="E30" s="11"/>
-      <c r="F30" s="12"/>
-      <c r="G30" s="12"/>
-      <c r="H30" s="10"/>
-      <c r="I30" s="10"/>
-      <c r="J30" s="10"/>
-      <c r="K30" s="10"/>
-      <c r="L30" s="10"/>
-      <c r="M30" s="10"/>
-      <c r="N30" s="10"/>
-      <c r="O30" s="10"/>
-      <c r="P30" s="10"/>
-      <c r="Q30" s="10"/>
-      <c r="R30" s="10"/>
-      <c r="S30" s="13">
-        <f>SUM(S6:S29)</f>
+    <row r="30">
+      <c r="A30" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B30" s="7">
+        <v>46181</v>
+      </c>
+      <c r="C30" s="7">
+        <v>46143</v>
+      </c>
+      <c r="D30" s="7">
+        <v>46181</v>
+      </c>
+      <c r="E30" s="7">
+        <v>46153</v>
+      </c>
+      <c r="F30" s="8">
+        <v>-1</v>
+      </c>
+      <c r="G30" s="8">
+        <v>-1</v>
+      </c>
+      <c r="H30" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="I30" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="J30" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="K30" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L30" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="M30" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="N30" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="O30" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="P30" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="Q30" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="R30" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="S30" s="9">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B31" s="7">
+        <v>46181</v>
+      </c>
+      <c r="C31" s="7">
+        <v>46143</v>
+      </c>
+      <c r="D31" s="7">
+        <v>46181</v>
+      </c>
+      <c r="E31" s="7">
+        <v>46167</v>
+      </c>
+      <c r="F31" s="8">
+        <v>-1</v>
+      </c>
+      <c r="G31" s="8">
+        <v>-1</v>
+      </c>
+      <c r="H31" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="I31" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="J31" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="K31" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L31" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="M31" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="N31" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="O31" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="P31" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q31" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="R31" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="S31" s="9">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B32" s="7">
+        <v>46181</v>
+      </c>
+      <c r="C32" s="7">
+        <v>46181</v>
+      </c>
+      <c r="D32" s="7">
+        <v>46181</v>
+      </c>
+      <c r="E32" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="F32" s="8">
+        <v>-1</v>
+      </c>
+      <c r="G32" s="8">
+        <v>-1</v>
+      </c>
+      <c r="H32" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="I32" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="J32" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="K32" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L32" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="M32" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="N32" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="O32" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="P32" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q32" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="R32" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="S32" s="9">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B33" s="7">
+        <v>46181</v>
+      </c>
+      <c r="C33" s="7">
+        <v>46181</v>
+      </c>
+      <c r="D33" s="7">
+        <v>46181</v>
+      </c>
+      <c r="E33" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="F33" s="8">
+        <v>-1</v>
+      </c>
+      <c r="G33" s="8">
+        <v>-1</v>
+      </c>
+      <c r="H33" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="I33" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="J33" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="K33" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L33" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="M33" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="N33" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="O33" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="P33" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q33" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="R33" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="S33" s="9">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B34" s="7">
+        <v>46181</v>
+      </c>
+      <c r="C34" s="7">
+        <v>46082</v>
+      </c>
+      <c r="D34" s="7">
+        <v>46181</v>
+      </c>
+      <c r="E34" s="7">
+        <v>46097</v>
+      </c>
+      <c r="F34" s="8">
+        <v>-1</v>
+      </c>
+      <c r="G34" s="8">
+        <v>-1</v>
+      </c>
+      <c r="H34" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="I34" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="J34" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="K34" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L34" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="M34" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="N34" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="O34" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="P34" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q34" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="R34" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="S34" s="9">
+        <v>146.55</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B35" s="7">
+        <v>46181</v>
+      </c>
+      <c r="C35" s="7">
+        <v>46181</v>
+      </c>
+      <c r="D35" s="7">
+        <v>46181</v>
+      </c>
+      <c r="E35" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="F35" s="8">
+        <v>-1</v>
+      </c>
+      <c r="G35" s="8">
+        <v>-1</v>
+      </c>
+      <c r="H35" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="I35" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="J35" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="K35" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L35" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="M35" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="N35" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="O35" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="P35" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q35" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="R35" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="S35" s="9">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B36" s="7">
+        <v>46181</v>
+      </c>
+      <c r="C36" s="7">
+        <v>46181</v>
+      </c>
+      <c r="D36" s="7">
+        <v>46181</v>
+      </c>
+      <c r="E36" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="F36" s="8">
+        <v>-1</v>
+      </c>
+      <c r="G36" s="8">
+        <v>-1</v>
+      </c>
+      <c r="H36" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="I36" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="J36" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="K36" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L36" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="M36" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="N36" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="O36" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="P36" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q36" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="R36" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="S36" s="9">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B37" s="7">
+        <v>46181</v>
+      </c>
+      <c r="C37" s="7">
+        <v>46181</v>
+      </c>
+      <c r="D37" s="7">
+        <v>46181</v>
+      </c>
+      <c r="E37" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="F37" s="8">
+        <v>-1</v>
+      </c>
+      <c r="G37" s="8">
+        <v>-1</v>
+      </c>
+      <c r="H37" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="I37" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="J37" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="K37" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L37" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="M37" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="N37" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="O37" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="P37" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q37" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="R37" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="S37" s="9">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B38" s="7">
+        <v>46181</v>
+      </c>
+      <c r="C38" s="7">
+        <v>46181</v>
+      </c>
+      <c r="D38" s="7">
+        <v>46181</v>
+      </c>
+      <c r="E38" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="F38" s="8">
+        <v>-1</v>
+      </c>
+      <c r="G38" s="8">
+        <v>-1</v>
+      </c>
+      <c r="H38" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="I38" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="J38" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="K38" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L38" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="M38" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="N38" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="O38" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="P38" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q38" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="R38" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="S38" s="9">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B39" s="7">
+        <v>46181</v>
+      </c>
+      <c r="C39" s="7">
+        <v>46167</v>
+      </c>
+      <c r="D39" s="7">
+        <v>46167</v>
+      </c>
+      <c r="E39" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="F39" s="8">
+        <v>-15</v>
+      </c>
+      <c r="G39" s="8">
+        <v>-1</v>
+      </c>
+      <c r="H39" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="I39" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="J39" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="K39" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L39" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="M39" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="N39" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="O39" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="P39" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q39" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="R39" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="S39" s="9">
+        <v>193.43</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B40" s="7">
+        <v>46181</v>
+      </c>
+      <c r="C40" s="7">
+        <v>46167</v>
+      </c>
+      <c r="D40" s="7">
+        <v>46167</v>
+      </c>
+      <c r="E40" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="F40" s="8">
+        <v>-15</v>
+      </c>
+      <c r="G40" s="8">
+        <v>-1</v>
+      </c>
+      <c r="H40" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="I40" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="J40" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="K40" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L40" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="M40" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="N40" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="O40" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="P40" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q40" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="R40" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="S40" s="9">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B41" s="7">
+        <v>46181</v>
+      </c>
+      <c r="C41" s="7">
+        <v>46174</v>
+      </c>
+      <c r="D41" s="7">
+        <v>46174</v>
+      </c>
+      <c r="E41" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="F41" s="8">
+        <v>-8</v>
+      </c>
+      <c r="G41" s="8">
+        <v>-1</v>
+      </c>
+      <c r="H41" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="I41" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="J41" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="K41" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L41" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="M41" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="N41" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="O41" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="P41" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q41" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="R41" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="S41" s="9">
+        <v>302.72</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B42" s="7">
+        <v>46181</v>
+      </c>
+      <c r="C42" s="7">
+        <v>46174</v>
+      </c>
+      <c r="D42" s="7">
+        <v>46174</v>
+      </c>
+      <c r="E42" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="F42" s="8">
+        <v>-8</v>
+      </c>
+      <c r="G42" s="8">
+        <v>-1</v>
+      </c>
+      <c r="H42" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="I42" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="J42" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="K42" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L42" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="M42" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="N42" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="O42" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="P42" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q42" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="R42" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="S42" s="9">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B43" s="7">
+        <v>46181</v>
+      </c>
+      <c r="C43" s="7">
+        <v>46174</v>
+      </c>
+      <c r="D43" s="7">
+        <v>46174</v>
+      </c>
+      <c r="E43" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="F43" s="8">
+        <v>-8</v>
+      </c>
+      <c r="G43" s="8">
+        <v>-1</v>
+      </c>
+      <c r="H43" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="I43" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="J43" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="K43" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L43" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="M43" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="N43" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="O43" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="P43" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q43" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="R43" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="S43" s="9">
+        <v>579.12</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B44" s="7">
+        <v>46181</v>
+      </c>
+      <c r="C44" s="7">
+        <v>46181</v>
+      </c>
+      <c r="D44" s="7">
+        <v>46181</v>
+      </c>
+      <c r="E44" s="7">
+        <v>46170</v>
+      </c>
+      <c r="F44" s="8">
+        <v>-1</v>
+      </c>
+      <c r="G44" s="8">
+        <v>-1</v>
+      </c>
+      <c r="H44" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="I44" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="J44" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="K44" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L44" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="M44" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="N44" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="O44" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="P44" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q44" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="R44" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="S44" s="9">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B45" s="7">
+        <v>46181</v>
+      </c>
+      <c r="C45" s="7">
+        <v>46181</v>
+      </c>
+      <c r="D45" s="7">
+        <v>46181</v>
+      </c>
+      <c r="E45" s="7">
+        <v>46141</v>
+      </c>
+      <c r="F45" s="8">
+        <v>-1</v>
+      </c>
+      <c r="G45" s="8">
+        <v>-1</v>
+      </c>
+      <c r="H45" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="I45" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="J45" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="K45" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L45" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="M45" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="N45" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="O45" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="P45" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q45" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="R45" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="S45" s="9">
+        <v>620</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B46" s="7">
+        <v>46181</v>
+      </c>
+      <c r="C46" s="7">
+        <v>46181</v>
+      </c>
+      <c r="D46" s="7">
+        <v>46181</v>
+      </c>
+      <c r="E46" s="7">
+        <v>46141</v>
+      </c>
+      <c r="F46" s="8">
+        <v>-1</v>
+      </c>
+      <c r="G46" s="8">
+        <v>-1</v>
+      </c>
+      <c r="H46" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="I46" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="J46" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="K46" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L46" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="M46" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="N46" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="O46" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="P46" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q46" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="R46" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="S46" s="9">
+        <v>620</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B47" s="7">
+        <v>46181</v>
+      </c>
+      <c r="C47" s="7">
+        <v>46181</v>
+      </c>
+      <c r="D47" s="7">
+        <v>46181</v>
+      </c>
+      <c r="E47" s="7">
+        <v>46170</v>
+      </c>
+      <c r="F47" s="8">
+        <v>-1</v>
+      </c>
+      <c r="G47" s="8">
+        <v>-1</v>
+      </c>
+      <c r="H47" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="I47" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="J47" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="K47" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L47" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="M47" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="N47" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="O47" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="P47" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q47" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="R47" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="S47" s="9">
+        <v>630</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B48" s="7">
+        <v>46181</v>
+      </c>
+      <c r="C48" s="7">
+        <v>46181</v>
+      </c>
+      <c r="D48" s="7">
+        <v>46181</v>
+      </c>
+      <c r="E48" s="7">
+        <v>46164</v>
+      </c>
+      <c r="F48" s="8">
+        <v>-1</v>
+      </c>
+      <c r="G48" s="8">
+        <v>-1</v>
+      </c>
+      <c r="H48" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="I48" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="J48" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="K48" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L48" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="M48" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="N48" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="O48" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="P48" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q48" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="R48" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="S48" s="9">
+        <v>630</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B49" s="7">
+        <v>46181</v>
+      </c>
+      <c r="C49" s="7">
+        <v>46181</v>
+      </c>
+      <c r="D49" s="7">
+        <v>46181</v>
+      </c>
+      <c r="E49" s="7">
+        <v>46169</v>
+      </c>
+      <c r="F49" s="8">
+        <v>-1</v>
+      </c>
+      <c r="G49" s="8">
+        <v>-1</v>
+      </c>
+      <c r="H49" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="I49" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="J49" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="K49" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L49" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="M49" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="N49" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="O49" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="P49" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q49" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="R49" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="S49" s="9">
+        <v>630</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B50" s="7">
+        <v>46181</v>
+      </c>
+      <c r="C50" s="7">
+        <v>46181</v>
+      </c>
+      <c r="D50" s="7">
+        <v>46181</v>
+      </c>
+      <c r="E50" s="7">
+        <v>46163</v>
+      </c>
+      <c r="F50" s="8">
+        <v>-1</v>
+      </c>
+      <c r="G50" s="8">
+        <v>-1</v>
+      </c>
+      <c r="H50" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="I50" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="J50" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="K50" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L50" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="M50" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="N50" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="O50" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="P50" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q50" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="R50" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="S50" s="9">
+        <v>630</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B51" s="7">
+        <v>46181</v>
+      </c>
+      <c r="C51" s="7">
+        <v>46181</v>
+      </c>
+      <c r="D51" s="7">
+        <v>46181</v>
+      </c>
+      <c r="E51" s="7">
+        <v>46170</v>
+      </c>
+      <c r="F51" s="8">
+        <v>-1</v>
+      </c>
+      <c r="G51" s="8">
+        <v>-1</v>
+      </c>
+      <c r="H51" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="I51" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="J51" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="K51" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L51" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="M51" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="N51" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="O51" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="P51" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q51" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="R51" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="S51" s="9">
+        <v>650</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B52" s="7">
+        <v>46181</v>
+      </c>
+      <c r="C52" s="7">
+        <v>46181</v>
+      </c>
+      <c r="D52" s="7">
+        <v>46181</v>
+      </c>
+      <c r="E52" s="7">
+        <v>46170</v>
+      </c>
+      <c r="F52" s="8">
+        <v>-1</v>
+      </c>
+      <c r="G52" s="8">
+        <v>-1</v>
+      </c>
+      <c r="H52" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="I52" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="J52" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="K52" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L52" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="M52" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="N52" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="O52" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="P52" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q52" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="R52" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="S52" s="9">
+        <v>650</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B53" s="7">
+        <v>46181</v>
+      </c>
+      <c r="C53" s="7">
+        <v>46181</v>
+      </c>
+      <c r="D53" s="7">
+        <v>46181</v>
+      </c>
+      <c r="E53" s="7">
+        <v>46167</v>
+      </c>
+      <c r="F53" s="8">
+        <v>-1</v>
+      </c>
+      <c r="G53" s="8">
+        <v>-1</v>
+      </c>
+      <c r="H53" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="I53" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="J53" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="K53" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L53" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="M53" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="N53" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="O53" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="P53" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q53" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="R53" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="S53" s="9">
+        <v>680</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B54" s="7">
+        <v>46181</v>
+      </c>
+      <c r="C54" s="7">
+        <v>46181</v>
+      </c>
+      <c r="D54" s="7">
+        <v>46181</v>
+      </c>
+      <c r="E54" s="7">
+        <v>46141</v>
+      </c>
+      <c r="F54" s="8">
+        <v>-1</v>
+      </c>
+      <c r="G54" s="8">
+        <v>-1</v>
+      </c>
+      <c r="H54" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="I54" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="J54" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="K54" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L54" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="M54" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="N54" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="O54" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="P54" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q54" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="R54" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="S54" s="9">
+        <v>680</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B55" s="7">
+        <v>46181</v>
+      </c>
+      <c r="C55" s="7">
+        <v>46181</v>
+      </c>
+      <c r="D55" s="7">
+        <v>46181</v>
+      </c>
+      <c r="E55" s="7">
+        <v>46182</v>
+      </c>
+      <c r="F55" s="8">
+        <v>-1</v>
+      </c>
+      <c r="G55" s="8">
+        <v>-1</v>
+      </c>
+      <c r="H55" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="I55" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="J55" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="K55" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L55" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="M55" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="N55" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="O55" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="P55" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q55" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="R55" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="S55" s="9">
+        <v>680</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B56" s="7">
+        <v>46181</v>
+      </c>
+      <c r="C56" s="7">
+        <v>46181</v>
+      </c>
+      <c r="D56" s="7">
+        <v>46181</v>
+      </c>
+      <c r="E56" s="7">
+        <v>46182</v>
+      </c>
+      <c r="F56" s="8">
+        <v>-1</v>
+      </c>
+      <c r="G56" s="8">
+        <v>-1</v>
+      </c>
+      <c r="H56" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="I56" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="J56" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="K56" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L56" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="M56" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="N56" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="O56" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="P56" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q56" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="R56" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="S56" s="9">
+        <v>680</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B57" s="7">
+        <v>46181</v>
+      </c>
+      <c r="C57" s="7">
+        <v>46181</v>
+      </c>
+      <c r="D57" s="7">
+        <v>46181</v>
+      </c>
+      <c r="E57" s="7">
+        <v>46164</v>
+      </c>
+      <c r="F57" s="8">
+        <v>-1</v>
+      </c>
+      <c r="G57" s="8">
+        <v>-1</v>
+      </c>
+      <c r="H57" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="I57" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="J57" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="K57" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L57" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="M57" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="N57" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="O57" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="P57" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q57" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="R57" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="S57" s="9">
+        <v>680</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B58" s="7">
+        <v>46181</v>
+      </c>
+      <c r="C58" s="7">
+        <v>46181</v>
+      </c>
+      <c r="D58" s="7">
+        <v>46181</v>
+      </c>
+      <c r="E58" s="7">
+        <v>46170</v>
+      </c>
+      <c r="F58" s="8">
+        <v>-1</v>
+      </c>
+      <c r="G58" s="8">
+        <v>-1</v>
+      </c>
+      <c r="H58" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="I58" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="J58" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="K58" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L58" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="M58" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="N58" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="O58" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="P58" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="Q58" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="R58" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="S58" s="9">
+        <v>700</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B59" s="7">
+        <v>46181</v>
+      </c>
+      <c r="C59" s="7">
+        <v>46181</v>
+      </c>
+      <c r="D59" s="7">
+        <v>46181</v>
+      </c>
+      <c r="E59" s="7">
+        <v>46170</v>
+      </c>
+      <c r="F59" s="8">
+        <v>-1</v>
+      </c>
+      <c r="G59" s="8">
+        <v>-1</v>
+      </c>
+      <c r="H59" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="I59" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="J59" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="K59" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L59" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="M59" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="N59" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="O59" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="P59" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q59" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="R59" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="S59" s="9">
+        <v>700</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="B60" s="7">
+        <v>46181</v>
+      </c>
+      <c r="C60" s="7">
+        <v>46181</v>
+      </c>
+      <c r="D60" s="7">
+        <v>46181</v>
+      </c>
+      <c r="E60" s="7">
+        <v>46182</v>
+      </c>
+      <c r="F60" s="8">
+        <v>-1</v>
+      </c>
+      <c r="G60" s="8">
+        <v>-1</v>
+      </c>
+      <c r="H60" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="I60" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="J60" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="K60" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L60" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="M60" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="N60" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="O60" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="P60" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q60" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="R60" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="S60" s="9">
+        <v>800</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B61" s="7">
+        <v>46181</v>
+      </c>
+      <c r="C61" s="7">
+        <v>46181</v>
+      </c>
+      <c r="D61" s="7">
+        <v>46181</v>
+      </c>
+      <c r="E61" s="7">
+        <v>46148</v>
+      </c>
+      <c r="F61" s="8">
+        <v>-1</v>
+      </c>
+      <c r="G61" s="8">
+        <v>-1</v>
+      </c>
+      <c r="H61" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="I61" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="J61" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="K61" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L61" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="M61" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="N61" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="O61" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="P61" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q61" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="R61" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="S61" s="9">
+        <v>800</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B62" s="7">
+        <v>46181</v>
+      </c>
+      <c r="C62" s="7">
+        <v>46181</v>
+      </c>
+      <c r="D62" s="7">
+        <v>46181</v>
+      </c>
+      <c r="E62" s="7">
+        <v>46148</v>
+      </c>
+      <c r="F62" s="8">
+        <v>-1</v>
+      </c>
+      <c r="G62" s="8">
+        <v>-1</v>
+      </c>
+      <c r="H62" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="I62" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="J62" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="K62" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L62" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="M62" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="N62" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="O62" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="P62" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q62" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="R62" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="S62" s="9">
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B63" s="7">
+        <v>46181</v>
+      </c>
+      <c r="C63" s="7">
+        <v>46143</v>
+      </c>
+      <c r="D63" s="7">
+        <v>46181</v>
+      </c>
+      <c r="E63" s="7">
+        <v>46170</v>
+      </c>
+      <c r="F63" s="8">
+        <v>-1</v>
+      </c>
+      <c r="G63" s="8">
+        <v>-1</v>
+      </c>
+      <c r="H63" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="I63" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="J63" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="K63" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L63" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="M63" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="N63" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="O63" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="P63" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q63" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="R63" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="S63" s="9">
+        <v>2969.17</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B64" s="7">
+        <v>46182</v>
+      </c>
+      <c r="C64" s="7">
+        <v>46181</v>
+      </c>
+      <c r="D64" s="7">
+        <v>46181</v>
+      </c>
+      <c r="E64" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="F64" s="8">
+        <v>-1</v>
+      </c>
+      <c r="G64" s="8">
+        <v>0</v>
+      </c>
+      <c r="H64" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="I64" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="J64" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="K64" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L64" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="M64" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="N64" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="O64" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="P64" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q64" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="R64" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="S64" s="9">
+        <v>215.07</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B65" s="7">
+        <v>46182</v>
+      </c>
+      <c r="C65" s="7">
+        <v>46181</v>
+      </c>
+      <c r="D65" s="7">
+        <v>46181</v>
+      </c>
+      <c r="E65" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="F65" s="8">
+        <v>-1</v>
+      </c>
+      <c r="G65" s="8">
+        <v>0</v>
+      </c>
+      <c r="H65" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="I65" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="J65" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="K65" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L65" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="M65" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="N65" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="O65" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="P65" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q65" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="R65" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="S65" s="9">
+        <v>237.36</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B66" s="7">
+        <v>46182</v>
+      </c>
+      <c r="C66" s="7">
+        <v>46181</v>
+      </c>
+      <c r="D66" s="7">
+        <v>46181</v>
+      </c>
+      <c r="E66" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="F66" s="8">
+        <v>-1</v>
+      </c>
+      <c r="G66" s="8">
+        <v>0</v>
+      </c>
+      <c r="H66" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="I66" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="J66" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="K66" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L66" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="M66" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="N66" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="O66" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="P66" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q66" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="R66" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="S66" s="9">
+        <v>431.06</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B67" s="7">
+        <v>46188</v>
+      </c>
+      <c r="C67" s="7">
+        <v>46143</v>
+      </c>
+      <c r="D67" s="7">
+        <v>46188</v>
+      </c>
+      <c r="E67" s="7">
+        <v>46153</v>
+      </c>
+      <c r="F67" s="8">
+        <v>6</v>
+      </c>
+      <c r="G67" s="8">
+        <v>6</v>
+      </c>
+      <c r="H67" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I67" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="J67" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="K67" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L67" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="M67" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="N67" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="O67" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="P67" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="Q67" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="R67" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="S67" s="9">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B68" s="7">
+        <v>46188</v>
+      </c>
+      <c r="C68" s="7">
+        <v>46143</v>
+      </c>
+      <c r="D68" s="7">
+        <v>46188</v>
+      </c>
+      <c r="E68" s="7">
+        <v>46167</v>
+      </c>
+      <c r="F68" s="8">
+        <v>6</v>
+      </c>
+      <c r="G68" s="8">
+        <v>6</v>
+      </c>
+      <c r="H68" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I68" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="J68" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="K68" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L68" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="M68" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="N68" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="O68" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="P68" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q68" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="R68" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="S68" s="9">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B69" s="7">
+        <v>46188</v>
+      </c>
+      <c r="C69" s="7">
+        <v>46188</v>
+      </c>
+      <c r="D69" s="7">
+        <v>46188</v>
+      </c>
+      <c r="E69" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="F69" s="8">
+        <v>6</v>
+      </c>
+      <c r="G69" s="8">
+        <v>6</v>
+      </c>
+      <c r="H69" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I69" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="J69" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="K69" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L69" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="M69" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="N69" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="O69" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="P69" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q69" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="R69" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="S69" s="9">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B70" s="7">
+        <v>46188</v>
+      </c>
+      <c r="C70" s="7">
+        <v>46082</v>
+      </c>
+      <c r="D70" s="7">
+        <v>46188</v>
+      </c>
+      <c r="E70" s="7">
+        <v>46097</v>
+      </c>
+      <c r="F70" s="8">
+        <v>6</v>
+      </c>
+      <c r="G70" s="8">
+        <v>6</v>
+      </c>
+      <c r="H70" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I70" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="J70" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="K70" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L70" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="M70" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="N70" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="O70" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="P70" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q70" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="R70" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="S70" s="9">
+        <v>146.55</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B71" s="7">
+        <v>46188</v>
+      </c>
+      <c r="C71" s="7">
+        <v>46188</v>
+      </c>
+      <c r="D71" s="7">
+        <v>46188</v>
+      </c>
+      <c r="E71" s="7">
+        <v>46169</v>
+      </c>
+      <c r="F71" s="8">
+        <v>6</v>
+      </c>
+      <c r="G71" s="8">
+        <v>6</v>
+      </c>
+      <c r="H71" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I71" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="J71" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="K71" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L71" s="6" t="s">
+        <v>116</v>
+      </c>
+      <c r="M71" s="6" t="s">
+        <v>116</v>
+      </c>
+      <c r="N71" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="O71" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="P71" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q71" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="R71" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="S71" s="9">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B72" s="7">
+        <v>46188</v>
+      </c>
+      <c r="C72" s="7">
+        <v>46188</v>
+      </c>
+      <c r="D72" s="7">
+        <v>46188</v>
+      </c>
+      <c r="E72" s="7">
+        <v>46170</v>
+      </c>
+      <c r="F72" s="8">
+        <v>6</v>
+      </c>
+      <c r="G72" s="8">
+        <v>6</v>
+      </c>
+      <c r="H72" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I72" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="J72" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="K72" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L72" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="M72" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="N72" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="O72" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="P72" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q72" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="R72" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="S72" s="9">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B73" s="7">
+        <v>46188</v>
+      </c>
+      <c r="C73" s="7">
+        <v>46188</v>
+      </c>
+      <c r="D73" s="7">
+        <v>46188</v>
+      </c>
+      <c r="E73" s="7">
+        <v>46169</v>
+      </c>
+      <c r="F73" s="8">
+        <v>6</v>
+      </c>
+      <c r="G73" s="8">
+        <v>6</v>
+      </c>
+      <c r="H73" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I73" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="J73" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="K73" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L73" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="M73" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="N73" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="O73" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="P73" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q73" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="R73" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="S73" s="9">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B74" s="7">
+        <v>46188</v>
+      </c>
+      <c r="C74" s="7">
+        <v>46188</v>
+      </c>
+      <c r="D74" s="7">
+        <v>46188</v>
+      </c>
+      <c r="E74" s="7">
+        <v>46141</v>
+      </c>
+      <c r="F74" s="8">
+        <v>6</v>
+      </c>
+      <c r="G74" s="8">
+        <v>6</v>
+      </c>
+      <c r="H74" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I74" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="J74" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="K74" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L74" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="M74" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="N74" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="O74" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="P74" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q74" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="R74" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="S74" s="9">
+        <v>620</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B75" s="7">
+        <v>46188</v>
+      </c>
+      <c r="C75" s="7">
+        <v>46188</v>
+      </c>
+      <c r="D75" s="7">
+        <v>46188</v>
+      </c>
+      <c r="E75" s="7">
+        <v>46176</v>
+      </c>
+      <c r="F75" s="8">
+        <v>6</v>
+      </c>
+      <c r="G75" s="8">
+        <v>6</v>
+      </c>
+      <c r="H75" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I75" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="J75" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="K75" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L75" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="M75" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="N75" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="O75" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="P75" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q75" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="R75" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="S75" s="9">
+        <v>620</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B76" s="7">
+        <v>46188</v>
+      </c>
+      <c r="C76" s="7">
+        <v>46188</v>
+      </c>
+      <c r="D76" s="7">
+        <v>46188</v>
+      </c>
+      <c r="E76" s="7">
+        <v>46141</v>
+      </c>
+      <c r="F76" s="8">
+        <v>6</v>
+      </c>
+      <c r="G76" s="8">
+        <v>6</v>
+      </c>
+      <c r="H76" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I76" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="J76" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="K76" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L76" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="M76" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="N76" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="O76" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="P76" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q76" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="R76" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="S76" s="9">
+        <v>620</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B77" s="7">
+        <v>46188</v>
+      </c>
+      <c r="C77" s="7">
+        <v>46188</v>
+      </c>
+      <c r="D77" s="7">
+        <v>46188</v>
+      </c>
+      <c r="E77" s="7">
+        <v>46170</v>
+      </c>
+      <c r="F77" s="8">
+        <v>6</v>
+      </c>
+      <c r="G77" s="8">
+        <v>6</v>
+      </c>
+      <c r="H77" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I77" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="J77" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="K77" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L77" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="M77" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="N77" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="O77" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="P77" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="Q77" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="R77" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="S77" s="9">
+        <v>630</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B78" s="7">
+        <v>46188</v>
+      </c>
+      <c r="C78" s="7">
+        <v>46188</v>
+      </c>
+      <c r="D78" s="7">
+        <v>46188</v>
+      </c>
+      <c r="E78" s="7">
+        <v>46170</v>
+      </c>
+      <c r="F78" s="8">
+        <v>6</v>
+      </c>
+      <c r="G78" s="8">
+        <v>6</v>
+      </c>
+      <c r="H78" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I78" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="J78" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="K78" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L78" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="M78" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="N78" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="O78" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="P78" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q78" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="R78" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="S78" s="9">
+        <v>630</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B79" s="7">
+        <v>46188</v>
+      </c>
+      <c r="C79" s="7">
+        <v>46188</v>
+      </c>
+      <c r="D79" s="7">
+        <v>46188</v>
+      </c>
+      <c r="E79" s="7">
+        <v>46164</v>
+      </c>
+      <c r="F79" s="8">
+        <v>6</v>
+      </c>
+      <c r="G79" s="8">
+        <v>6</v>
+      </c>
+      <c r="H79" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I79" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="J79" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="K79" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L79" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="M79" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="N79" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="O79" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="P79" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q79" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="R79" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="S79" s="9">
+        <v>630</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B80" s="7">
+        <v>46188</v>
+      </c>
+      <c r="C80" s="7">
+        <v>46188</v>
+      </c>
+      <c r="D80" s="7">
+        <v>46188</v>
+      </c>
+      <c r="E80" s="7">
+        <v>46169</v>
+      </c>
+      <c r="F80" s="8">
+        <v>6</v>
+      </c>
+      <c r="G80" s="8">
+        <v>6</v>
+      </c>
+      <c r="H80" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I80" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="J80" s="6" t="s">
+        <v>126</v>
+      </c>
+      <c r="K80" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L80" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="M80" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="N80" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="O80" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="P80" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q80" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="R80" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="S80" s="9">
+        <v>630</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B81" s="7">
+        <v>46188</v>
+      </c>
+      <c r="C81" s="7">
+        <v>46188</v>
+      </c>
+      <c r="D81" s="7">
+        <v>46188</v>
+      </c>
+      <c r="E81" s="7">
+        <v>46163</v>
+      </c>
+      <c r="F81" s="8">
+        <v>6</v>
+      </c>
+      <c r="G81" s="8">
+        <v>6</v>
+      </c>
+      <c r="H81" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I81" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="J81" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="K81" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L81" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="M81" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="N81" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="O81" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="P81" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q81" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="R81" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="S81" s="9">
+        <v>630</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B82" s="7">
+        <v>46188</v>
+      </c>
+      <c r="C82" s="7">
+        <v>46188</v>
+      </c>
+      <c r="D82" s="7">
+        <v>46188</v>
+      </c>
+      <c r="E82" s="7">
+        <v>46169</v>
+      </c>
+      <c r="F82" s="8">
+        <v>6</v>
+      </c>
+      <c r="G82" s="8">
+        <v>6</v>
+      </c>
+      <c r="H82" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I82" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="J82" s="6" t="s">
+        <v>128</v>
+      </c>
+      <c r="K82" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L82" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="M82" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="N82" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="O82" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="P82" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q82" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="R82" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="S82" s="9">
+        <v>630</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B83" s="7">
+        <v>46188</v>
+      </c>
+      <c r="C83" s="7">
+        <v>46188</v>
+      </c>
+      <c r="D83" s="7">
+        <v>46188</v>
+      </c>
+      <c r="E83" s="7">
+        <v>46169</v>
+      </c>
+      <c r="F83" s="8">
+        <v>6</v>
+      </c>
+      <c r="G83" s="8">
+        <v>6</v>
+      </c>
+      <c r="H83" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I83" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="J83" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="K83" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L83" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="M83" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="N83" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="O83" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="P83" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q83" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="R83" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="S83" s="9">
+        <v>630</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B84" s="7">
+        <v>46188</v>
+      </c>
+      <c r="C84" s="7">
+        <v>46188</v>
+      </c>
+      <c r="D84" s="7">
+        <v>46188</v>
+      </c>
+      <c r="E84" s="7">
+        <v>46169</v>
+      </c>
+      <c r="F84" s="8">
+        <v>6</v>
+      </c>
+      <c r="G84" s="8">
+        <v>6</v>
+      </c>
+      <c r="H84" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I84" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="J84" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="K84" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L84" s="6" t="s">
+        <v>132</v>
+      </c>
+      <c r="M84" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="N84" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="O84" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="P84" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q84" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="R84" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="S84" s="9">
+        <v>630</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B85" s="7">
+        <v>46188</v>
+      </c>
+      <c r="C85" s="7">
+        <v>46188</v>
+      </c>
+      <c r="D85" s="7">
+        <v>46188</v>
+      </c>
+      <c r="E85" s="7">
+        <v>46170</v>
+      </c>
+      <c r="F85" s="8">
+        <v>6</v>
+      </c>
+      <c r="G85" s="8">
+        <v>6</v>
+      </c>
+      <c r="H85" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I85" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="J85" s="6" t="s">
+        <v>133</v>
+      </c>
+      <c r="K85" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L85" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="M85" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="N85" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="O85" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="P85" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q85" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="R85" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="S85" s="9">
+        <v>650</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B86" s="7">
+        <v>46188</v>
+      </c>
+      <c r="C86" s="7">
+        <v>46188</v>
+      </c>
+      <c r="D86" s="7">
+        <v>46188</v>
+      </c>
+      <c r="E86" s="7">
+        <v>46160</v>
+      </c>
+      <c r="F86" s="8">
+        <v>6</v>
+      </c>
+      <c r="G86" s="8">
+        <v>6</v>
+      </c>
+      <c r="H86" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I86" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="J86" s="6" t="s">
+        <v>134</v>
+      </c>
+      <c r="K86" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L86" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="M86" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="N86" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="O86" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="P86" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q86" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="R86" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="S86" s="9">
+        <v>650</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B87" s="7">
+        <v>46188</v>
+      </c>
+      <c r="C87" s="7">
+        <v>46188</v>
+      </c>
+      <c r="D87" s="7">
+        <v>46188</v>
+      </c>
+      <c r="E87" s="7">
+        <v>46153</v>
+      </c>
+      <c r="F87" s="8">
+        <v>6</v>
+      </c>
+      <c r="G87" s="8">
+        <v>6</v>
+      </c>
+      <c r="H87" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I87" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="J87" s="6" t="s">
+        <v>136</v>
+      </c>
+      <c r="K87" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L87" s="6" t="s">
+        <v>137</v>
+      </c>
+      <c r="M87" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="N87" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="O87" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="P87" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q87" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="R87" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="S87" s="9">
+        <v>650</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B88" s="7">
+        <v>46188</v>
+      </c>
+      <c r="C88" s="7">
+        <v>46188</v>
+      </c>
+      <c r="D88" s="7">
+        <v>46188</v>
+      </c>
+      <c r="E88" s="7">
+        <v>46170</v>
+      </c>
+      <c r="F88" s="8">
+        <v>6</v>
+      </c>
+      <c r="G88" s="8">
+        <v>6</v>
+      </c>
+      <c r="H88" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I88" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="J88" s="6" t="s">
+        <v>138</v>
+      </c>
+      <c r="K88" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L88" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="M88" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="N88" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="O88" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="P88" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q88" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="R88" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="S88" s="9">
+        <v>650</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B89" s="7">
+        <v>46188</v>
+      </c>
+      <c r="C89" s="7">
+        <v>46188</v>
+      </c>
+      <c r="D89" s="7">
+        <v>46188</v>
+      </c>
+      <c r="E89" s="7">
+        <v>46127</v>
+      </c>
+      <c r="F89" s="8">
+        <v>6</v>
+      </c>
+      <c r="G89" s="8">
+        <v>6</v>
+      </c>
+      <c r="H89" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I89" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="J89" s="6" t="s">
+        <v>139</v>
+      </c>
+      <c r="K89" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L89" s="6" t="s">
+        <v>140</v>
+      </c>
+      <c r="M89" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="N89" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="O89" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="P89" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q89" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="R89" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="S89" s="9">
+        <v>650</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B90" s="7">
+        <v>46188</v>
+      </c>
+      <c r="C90" s="7">
+        <v>46188</v>
+      </c>
+      <c r="D90" s="7">
+        <v>46188</v>
+      </c>
+      <c r="E90" s="7">
+        <v>46119</v>
+      </c>
+      <c r="F90" s="8">
+        <v>6</v>
+      </c>
+      <c r="G90" s="8">
+        <v>6</v>
+      </c>
+      <c r="H90" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I90" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="J90" s="6" t="s">
+        <v>141</v>
+      </c>
+      <c r="K90" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L90" s="6" t="s">
+        <v>142</v>
+      </c>
+      <c r="M90" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="N90" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="O90" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="P90" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q90" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="R90" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="S90" s="9">
+        <v>670</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B91" s="7">
+        <v>46188</v>
+      </c>
+      <c r="C91" s="7">
+        <v>46188</v>
+      </c>
+      <c r="D91" s="7">
+        <v>46188</v>
+      </c>
+      <c r="E91" s="7">
+        <v>46167</v>
+      </c>
+      <c r="F91" s="8">
+        <v>6</v>
+      </c>
+      <c r="G91" s="8">
+        <v>6</v>
+      </c>
+      <c r="H91" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I91" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="J91" s="6" t="s">
+        <v>143</v>
+      </c>
+      <c r="K91" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L91" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="M91" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="N91" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="O91" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="P91" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q91" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="R91" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="S91" s="9">
+        <v>680</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B92" s="7">
+        <v>46188</v>
+      </c>
+      <c r="C92" s="7">
+        <v>46188</v>
+      </c>
+      <c r="D92" s="7">
+        <v>46188</v>
+      </c>
+      <c r="E92" s="7">
+        <v>46176</v>
+      </c>
+      <c r="F92" s="8">
+        <v>6</v>
+      </c>
+      <c r="G92" s="8">
+        <v>6</v>
+      </c>
+      <c r="H92" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I92" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="J92" s="6" t="s">
+        <v>144</v>
+      </c>
+      <c r="K92" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L92" s="6" t="s">
+        <v>145</v>
+      </c>
+      <c r="M92" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="N92" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="O92" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="P92" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q92" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="R92" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="S92" s="9">
+        <v>680</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B93" s="7">
+        <v>46188</v>
+      </c>
+      <c r="C93" s="7">
+        <v>46188</v>
+      </c>
+      <c r="D93" s="7">
+        <v>46188</v>
+      </c>
+      <c r="E93" s="7">
+        <v>46182</v>
+      </c>
+      <c r="F93" s="8">
+        <v>6</v>
+      </c>
+      <c r="G93" s="8">
+        <v>6</v>
+      </c>
+      <c r="H93" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I93" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="J93" s="6" t="s">
+        <v>146</v>
+      </c>
+      <c r="K93" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L93" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="M93" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="N93" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="O93" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="P93" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q93" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="R93" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="S93" s="9">
+        <v>680</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B94" s="7">
+        <v>46188</v>
+      </c>
+      <c r="C94" s="7">
+        <v>46188</v>
+      </c>
+      <c r="D94" s="7">
+        <v>46188</v>
+      </c>
+      <c r="E94" s="7">
+        <v>46141</v>
+      </c>
+      <c r="F94" s="8">
+        <v>6</v>
+      </c>
+      <c r="G94" s="8">
+        <v>6</v>
+      </c>
+      <c r="H94" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I94" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="J94" s="6" t="s">
+        <v>147</v>
+      </c>
+      <c r="K94" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L94" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="M94" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="N94" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="O94" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="P94" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q94" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="R94" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="S94" s="9">
+        <v>680</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B95" s="7">
+        <v>46188</v>
+      </c>
+      <c r="C95" s="7">
+        <v>46188</v>
+      </c>
+      <c r="D95" s="7">
+        <v>46188</v>
+      </c>
+      <c r="E95" s="7">
+        <v>46182</v>
+      </c>
+      <c r="F95" s="8">
+        <v>6</v>
+      </c>
+      <c r="G95" s="8">
+        <v>6</v>
+      </c>
+      <c r="H95" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I95" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="J95" s="6" t="s">
+        <v>148</v>
+      </c>
+      <c r="K95" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L95" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="M95" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="N95" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="O95" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="P95" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q95" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="R95" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="S95" s="9">
+        <v>680</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B96" s="7">
+        <v>46188</v>
+      </c>
+      <c r="C96" s="7">
+        <v>46188</v>
+      </c>
+      <c r="D96" s="7">
+        <v>46188</v>
+      </c>
+      <c r="E96" s="7">
+        <v>46164</v>
+      </c>
+      <c r="F96" s="8">
+        <v>6</v>
+      </c>
+      <c r="G96" s="8">
+        <v>6</v>
+      </c>
+      <c r="H96" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I96" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="J96" s="6" t="s">
+        <v>149</v>
+      </c>
+      <c r="K96" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L96" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="M96" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="N96" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="O96" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="P96" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q96" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="R96" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="S96" s="9">
+        <v>680</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B97" s="7">
+        <v>46188</v>
+      </c>
+      <c r="C97" s="7">
+        <v>46188</v>
+      </c>
+      <c r="D97" s="7">
+        <v>46188</v>
+      </c>
+      <c r="E97" s="7">
+        <v>46182</v>
+      </c>
+      <c r="F97" s="8">
+        <v>6</v>
+      </c>
+      <c r="G97" s="8">
+        <v>6</v>
+      </c>
+      <c r="H97" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I97" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="J97" s="6" t="s">
+        <v>150</v>
+      </c>
+      <c r="K97" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L97" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="M97" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="N97" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="O97" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="P97" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q97" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="R97" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="S97" s="9">
+        <v>680</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B98" s="7">
+        <v>46188</v>
+      </c>
+      <c r="C98" s="7">
+        <v>46188</v>
+      </c>
+      <c r="D98" s="7">
+        <v>46188</v>
+      </c>
+      <c r="E98" s="7">
+        <v>46170</v>
+      </c>
+      <c r="F98" s="8">
+        <v>6</v>
+      </c>
+      <c r="G98" s="8">
+        <v>6</v>
+      </c>
+      <c r="H98" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I98" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="J98" s="6" t="s">
+        <v>151</v>
+      </c>
+      <c r="K98" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L98" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="M98" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="N98" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="O98" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="P98" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="Q98" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="R98" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="S98" s="9">
+        <v>700</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B99" s="7">
+        <v>46188</v>
+      </c>
+      <c r="C99" s="7">
+        <v>46188</v>
+      </c>
+      <c r="D99" s="7">
+        <v>46188</v>
+      </c>
+      <c r="E99" s="7">
+        <v>46170</v>
+      </c>
+      <c r="F99" s="8">
+        <v>6</v>
+      </c>
+      <c r="G99" s="8">
+        <v>6</v>
+      </c>
+      <c r="H99" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I99" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="J99" s="6" t="s">
+        <v>152</v>
+      </c>
+      <c r="K99" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L99" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="M99" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="N99" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="O99" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="P99" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q99" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="R99" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="S99" s="9">
+        <v>700</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B100" s="7">
+        <v>46188</v>
+      </c>
+      <c r="C100" s="7">
+        <v>46188</v>
+      </c>
+      <c r="D100" s="7">
+        <v>46188</v>
+      </c>
+      <c r="E100" s="7">
+        <v>46148</v>
+      </c>
+      <c r="F100" s="8">
+        <v>6</v>
+      </c>
+      <c r="G100" s="8">
+        <v>6</v>
+      </c>
+      <c r="H100" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I100" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="J100" s="6" t="s">
+        <v>153</v>
+      </c>
+      <c r="K100" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L100" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="M100" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="N100" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="O100" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="P100" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q100" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="R100" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="S100" s="9">
+        <v>800</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="B101" s="7">
+        <v>46188</v>
+      </c>
+      <c r="C101" s="7">
+        <v>46188</v>
+      </c>
+      <c r="D101" s="7">
+        <v>46188</v>
+      </c>
+      <c r="E101" s="7">
+        <v>46182</v>
+      </c>
+      <c r="F101" s="8">
+        <v>6</v>
+      </c>
+      <c r="G101" s="8">
+        <v>6</v>
+      </c>
+      <c r="H101" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I101" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="J101" s="6" t="s">
+        <v>154</v>
+      </c>
+      <c r="K101" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L101" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="M101" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="N101" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="O101" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="P101" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q101" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="R101" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="S101" s="9">
+        <v>800</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B102" s="7">
+        <v>46188</v>
+      </c>
+      <c r="C102" s="7">
+        <v>46188</v>
+      </c>
+      <c r="D102" s="7">
+        <v>46188</v>
+      </c>
+      <c r="E102" s="7">
+        <v>46148</v>
+      </c>
+      <c r="F102" s="8">
+        <v>6</v>
+      </c>
+      <c r="G102" s="8">
+        <v>6</v>
+      </c>
+      <c r="H102" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I102" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="J102" s="6" t="s">
+        <v>155</v>
+      </c>
+      <c r="K102" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L102" s="6" t="s">
+        <v>156</v>
+      </c>
+      <c r="M102" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="N102" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="O102" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="P102" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q102" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="R102" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="S102" s="9">
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B103" s="7">
+        <v>46188</v>
+      </c>
+      <c r="C103" s="7">
+        <v>46188</v>
+      </c>
+      <c r="D103" s="7">
+        <v>46188</v>
+      </c>
+      <c r="E103" s="7">
+        <v>46160</v>
+      </c>
+      <c r="F103" s="8">
+        <v>6</v>
+      </c>
+      <c r="G103" s="8">
+        <v>6</v>
+      </c>
+      <c r="H103" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I103" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="J103" s="6" t="s">
+        <v>157</v>
+      </c>
+      <c r="K103" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L103" s="6" t="s">
+        <v>158</v>
+      </c>
+      <c r="M103" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="N103" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="O103" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="P103" s="6" t="s">
+        <v>159</v>
+      </c>
+      <c r="Q103" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="R103" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="S103" s="9">
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B104" s="7">
+        <v>46188</v>
+      </c>
+      <c r="C104" s="7">
+        <v>46188</v>
+      </c>
+      <c r="D104" s="7">
+        <v>46188</v>
+      </c>
+      <c r="E104" s="7">
+        <v>46148</v>
+      </c>
+      <c r="F104" s="8">
+        <v>6</v>
+      </c>
+      <c r="G104" s="8">
+        <v>6</v>
+      </c>
+      <c r="H104" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I104" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="J104" s="6" t="s">
+        <v>160</v>
+      </c>
+      <c r="K104" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L104" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="M104" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="N104" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="O104" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="P104" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q104" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="R104" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="S104" s="9">
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B105" s="7">
+        <v>46188</v>
+      </c>
+      <c r="C105" s="7">
+        <v>46188</v>
+      </c>
+      <c r="D105" s="7">
+        <v>46188</v>
+      </c>
+      <c r="E105" s="7">
+        <v>46160</v>
+      </c>
+      <c r="F105" s="8">
+        <v>6</v>
+      </c>
+      <c r="G105" s="8">
+        <v>6</v>
+      </c>
+      <c r="H105" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I105" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="J105" s="6" t="s">
+        <v>161</v>
+      </c>
+      <c r="K105" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="L105" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="M105" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="N105" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="O105" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="P105" s="6" t="s">
+        <v>159</v>
+      </c>
+      <c r="Q105" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="R105" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="S105" s="9">
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="106" ht="23" customHeight="1">
+      <c r="A106" s="10"/>
+      <c r="B106" s="11"/>
+      <c r="C106" s="11"/>
+      <c r="D106" s="11"/>
+      <c r="E106" s="11"/>
+      <c r="F106" s="12"/>
+      <c r="G106" s="12"/>
+      <c r="H106" s="10"/>
+      <c r="I106" s="10"/>
+      <c r="J106" s="10"/>
+      <c r="K106" s="10"/>
+      <c r="L106" s="10"/>
+      <c r="M106" s="10"/>
+      <c r="N106" s="10"/>
+      <c r="O106" s="10"/>
+      <c r="P106" s="10"/>
+      <c r="Q106" s="10"/>
+      <c r="R106" s="10"/>
+      <c r="S106" s="13">
+        <f>SUM(S6:S105)</f>
       </c>
     </row>
   </sheetData>

</xml_diff>